<commit_message>
Run 1st code coverage
</commit_message>
<xml_diff>
--- a/test-cases/test-cases.xlsx
+++ b/test-cases/test-cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Library_Project3\Library_Project3\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E245D16-4CA1-471C-B2C0-6E19FFB2FF1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{337708DA-09A3-474B-ABAD-FE00BF93961C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="251">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -48,12 +48,6 @@
     <t>Test Steps</t>
   </si>
   <si>
-    <t>Expected Results</t>
-  </si>
-  <si>
-    <t>Actual Results</t>
-  </si>
-  <si>
     <t>Status</t>
   </si>
   <si>
@@ -75,9 +69,6 @@
     <t>อยู่หน้า Login, บัญชี admin มีอยู่จริง</t>
   </si>
   <si>
-    <t>User: adminPass: wrong123</t>
-  </si>
-  <si>
     <t>1. ไปที่หน้า Login2. กรอก Username3. กรอก Password ผิด4. คลิก Login</t>
   </si>
   <si>
@@ -105,9 +96,6 @@
     <t>อยู่หน้า Login, สถานะ Logged out</t>
   </si>
   <si>
-    <t>User: ' OR '1'='1Pass: any</t>
-  </si>
-  <si>
     <t>1. ไปที่หน้า Login2. กรอก SQLi Payload ใน Username3. กรอกรหัสผ่านมั่ว4. คลิก Login</t>
   </si>
   <si>
@@ -766,13 +754,37 @@
   </si>
   <si>
     <t>รหัสผ่านยังคงเป็นรหัสเดิม</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>ผลที่เกิดขึ้น</t>
+  </si>
+  <si>
+    <t>ผลที่คาดหวัง</t>
+  </si>
+  <si>
+    <t>เข้าสู่ระบบไม่ได้และแจ้งว่า Invalid username or password</t>
+  </si>
+  <si>
+    <t>ระบบมี Validation ตรวจสอบฟิลด์บังคับ และไม่รับค่าสคริปต์ที่กรอกเข้าไป โดยแจ้งเตือนให้กรอกข้อมูลให้ครบถ้วนก่อนบันทึก</t>
+  </si>
+  <si>
+    <t>User: admin Pass: wrong123</t>
+  </si>
+  <si>
+    <t>User: ' OR '1'='1 Pass: any</t>
+  </si>
+  <si>
+    <t>ล็อคอินไม่สำเร็จ</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -785,6 +797,20 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -794,7 +820,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -802,39 +828,459 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="19">
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
     <dxf>
       <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
-          <color rgb="FF356854"/>
+          <color indexed="64"/>
         </left>
         <right style="thin">
-          <color rgb="FF356854"/>
+          <color indexed="64"/>
         </right>
         <top style="thin">
-          <color rgb="FF356854"/>
+          <color indexed="64"/>
         </top>
         <bottom style="thin">
-          <color rgb="FF356854"/>
+          <color indexed="64"/>
         </bottom>
       </border>
     </dxf>
@@ -862,13 +1308,29 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF356854"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF356854"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF356854"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF356854"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="1">
     <tableStyle name="รวม 30 Test Case Design-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="0"/>
-      <tableStyleElement type="headerRow" dxfId="3"/>
-      <tableStyleElement type="firstRowStripe" dxfId="2"/>
-      <tableStyleElement type="secondRowStripe" dxfId="1"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="18"/>
+      <tableStyleElement type="headerRow" dxfId="17"/>
+      <tableStyleElement type="firstRowStripe" dxfId="16"/>
+      <tableStyleElement type="secondRowStripe" dxfId="15"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -887,19 +1349,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Security_Test_Cases" displayName="Security_Test_Cases" ref="A1:K31">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Security_Test_Cases" displayName="Security_Test_Cases" ref="A1:K31" headerRowDxfId="1" totalsRowDxfId="0" headerRowBorderDxfId="13" tableBorderDxfId="14">
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Test Case ID"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Test Case Title"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Priority"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Preconditions"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Test Data"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Test Steps"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Expected Results"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Actual Results"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Status"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Postconditions"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Test Case ID" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Test Case Title" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Priority" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Preconditions" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Test Data" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Test Steps" dataDxfId="6"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="ผลที่คาดหวัง" dataDxfId="5"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="ผลที่เกิดขึ้น" dataDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Status" dataDxfId="3"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Postconditions" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="รวม 30 Test Case Design-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1111,1007 +1573,1044 @@
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="28.28515625" customWidth="1"/>
-    <col min="3" max="3" width="35.42578125" customWidth="1"/>
+    <col min="3" max="3" width="44.5703125" customWidth="1"/>
     <col min="4" max="4" width="13.85546875" customWidth="1"/>
     <col min="5" max="5" width="28.42578125" customWidth="1"/>
-    <col min="6" max="8" width="37.5703125" customWidth="1"/>
-    <col min="9" max="9" width="16.140625" customWidth="1"/>
-    <col min="11" max="11" width="31.85546875" customWidth="1"/>
+    <col min="6" max="7" width="37.5703125" customWidth="1"/>
+    <col min="8" max="8" width="103.42578125" customWidth="1"/>
+    <col min="9" max="9" width="55.5703125" customWidth="1"/>
+    <col min="11" max="11" width="36" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="11" t="s">
+        <v>245</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>244</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="B2" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+      <c r="C2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="D2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="F2" s="13" t="s">
+        <v>248</v>
+      </c>
+      <c r="G2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="H2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="I2" s="12" t="s">
+        <v>246</v>
+      </c>
+      <c r="J2" s="13" t="s">
+        <v>243</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>249</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" s="12" t="s">
+        <v>250</v>
+      </c>
+      <c r="J3" s="13" t="s">
+        <v>243</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="I4" s="5"/>
+      <c r="J4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
+      <c r="K4" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K4" s="2" t="s">
+      <c r="E5" s="4" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
+      <c r="F5" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="G5" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="H5" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E5" s="2" t="s">
+      <c r="I5" s="15" t="s">
+        <v>247</v>
+      </c>
+      <c r="J5" s="13" t="s">
+        <v>243</v>
+      </c>
+      <c r="K5" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F5" s="2" t="s">
+    </row>
+    <row r="6" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="B6" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="C6" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="J5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K5" s="2" t="s">
+      <c r="D6" s="4" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
+      <c r="E6" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="G6" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="H6" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="I6" s="5"/>
+      <c r="J6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K6" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F6" s="2" t="s">
+    </row>
+    <row r="7" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="B7" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="C7" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="J6" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K6" s="2" t="s">
+      <c r="D7" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="2" t="s">
+      <c r="F7" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="G7" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="H7" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E7" s="2" t="s">
+      <c r="I7" s="5"/>
+      <c r="J7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K7" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="F7" s="2" t="s">
+    </row>
+    <row r="8" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="B8" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="C8" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="J7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K7" s="2" t="s">
+      <c r="D8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
+      <c r="F8" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="G8" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="H8" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E8" s="2" t="s">
+      <c r="I8" s="5"/>
+      <c r="J8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K8" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="F8" s="2" t="s">
+    </row>
+    <row r="9" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="B9" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="C9" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="J8" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K8" s="2" t="s">
+      <c r="D9" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="4" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="2" t="s">
+      <c r="F9" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="G9" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="H9" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="D9" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E9" s="2" t="s">
+      <c r="I9" s="5"/>
+      <c r="J9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K9" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="F9" s="2" t="s">
+    </row>
+    <row r="10" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="B10" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="C10" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="J9" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K9" s="2" t="s">
+      <c r="D10" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
+      <c r="F10" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="G10" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="H10" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E10" s="2" t="s">
+      <c r="I10" s="5"/>
+      <c r="J10" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K10" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="F10" s="2" t="s">
+    </row>
+    <row r="11" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="B11" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="C11" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="J10" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K10" s="2" t="s">
+      <c r="D11" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="4" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
+      <c r="F11" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="G11" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="H11" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E11" s="2" t="s">
+      <c r="I11" s="5"/>
+      <c r="J11" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K11" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="F11" s="2" t="s">
+    </row>
+    <row r="12" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="B12" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="C12" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="J11" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K11" s="2" t="s">
+      <c r="D12" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" s="4" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="2" t="s">
+      <c r="F12" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="G12" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="H12" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E12" s="2" t="s">
+      <c r="I12" s="5"/>
+      <c r="J12" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K12" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="F12" s="2" t="s">
+    </row>
+    <row r="13" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="B13" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="C13" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="J12" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K12" s="2" t="s">
+      <c r="D13" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E13" s="4" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="2" t="s">
+      <c r="F13" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="G13" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="H13" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="D13" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E13" s="2" t="s">
+      <c r="I13" s="5"/>
+      <c r="J13" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K13" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="F13" s="2" t="s">
+    </row>
+    <row r="14" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="B14" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="H13" s="2" t="s">
+      <c r="C14" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="J13" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K13" s="2" t="s">
+      <c r="D14" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E14" s="4" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="2" t="s">
+      <c r="F14" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="G14" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="H14" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E14" s="2" t="s">
+      <c r="I14" s="5"/>
+      <c r="J14" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K14" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="F14" s="2" t="s">
+    </row>
+    <row r="15" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="B15" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="H14" s="2" t="s">
+      <c r="C15" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="J14" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K14" s="2" t="s">
+      <c r="D15" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="F15" s="4" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="2" t="s">
+      <c r="G15" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="H15" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="I15" s="5"/>
+      <c r="J15" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K15" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="D15" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="F15" s="2" t="s">
+    </row>
+    <row r="16" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="B16" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="C16" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="J15" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K15" s="2" t="s">
+      <c r="D16" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="F16" s="4" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="2" t="s">
+      <c r="G16" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="H16" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="I16" s="5"/>
+      <c r="J16" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K16" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="D16" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="F16" s="2" t="s">
+    </row>
+    <row r="17" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="B17" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="H16" s="2" t="s">
+      <c r="C17" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="J16" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K16" s="2" t="s">
+      <c r="D17" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" s="4" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="2" t="s">
+      <c r="F17" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="G17" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="H17" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I17" s="5"/>
+      <c r="J17" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K17" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="D17" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E17" s="2" t="s">
+    </row>
+    <row r="18" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="B18" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="G17" s="2" t="s">
+      <c r="C18" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="H17" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K17" s="2" t="s">
+      <c r="D18" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E18" s="4" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="2" t="s">
+      <c r="F18" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="G18" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="H18" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="D18" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E18" s="2" t="s">
+      <c r="I18" s="5"/>
+      <c r="J18" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K18" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="F18" s="2" t="s">
+    </row>
+    <row r="19" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="G18" s="2" t="s">
+      <c r="B19" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="H18" s="2" t="s">
+      <c r="C19" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="J18" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K18" s="2" t="s">
+      <c r="D19" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="F19" s="4" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="2" t="s">
+      <c r="G19" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="H19" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="I19" s="5"/>
+      <c r="J19" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K19" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="D19" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="F19" s="2" t="s">
+    </row>
+    <row r="20" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="B20" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="C20" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="J19" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K19" s="2" t="s">
+      <c r="D20" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="F20" s="4" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="2" t="s">
+      <c r="G20" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="H20" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="I20" s="5"/>
+      <c r="J20" s="13" t="s">
+        <v>243</v>
+      </c>
+      <c r="K20" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="D20" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="F20" s="2" t="s">
+    </row>
+    <row r="21" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="G20" s="2" t="s">
+      <c r="B21" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="H20" s="2" t="s">
+      <c r="C21" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="J20" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K20" s="2" t="s">
+      <c r="D21" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" s="4" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="2" t="s">
+      <c r="F21" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="G21" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="H21" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="D21" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E21" s="2" t="s">
+      <c r="I21" s="5"/>
+      <c r="J21" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K21" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="F21" s="2" t="s">
+    </row>
+    <row r="22" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="G21" s="2" t="s">
+      <c r="B22" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="H21" s="2" t="s">
+      <c r="C22" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="J21" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K21" s="2" t="s">
+      <c r="D22" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E22" s="4" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="2" t="s">
+      <c r="F22" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="G22" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="H22" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="D22" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E22" s="2" t="s">
+      <c r="I22" s="5"/>
+      <c r="J22" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K22" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="F22" s="2" t="s">
+    </row>
+    <row r="23" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="G22" s="2" t="s">
+      <c r="B23" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="H22" s="2" t="s">
+      <c r="C23" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="J22" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K22" s="2" t="s">
+      <c r="D23" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F23" s="4" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="2" t="s">
+      <c r="G23" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="H23" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="I23" s="5"/>
+      <c r="J23" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K23" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="D23" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="F23" s="2" t="s">
+    </row>
+    <row r="24" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="G23" s="2" t="s">
+      <c r="B24" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="H23" s="2" t="s">
+      <c r="C24" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="J23" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K23" s="2" t="s">
+      <c r="D24" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" s="4" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="24" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="2" t="s">
+      <c r="F24" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="G24" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="H24" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="D24" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E24" s="2" t="s">
+      <c r="I24" s="5"/>
+      <c r="J24" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K24" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="F24" s="2" t="s">
+    </row>
+    <row r="25" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="G24" s="2" t="s">
+      <c r="B25" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="H24" s="2" t="s">
+      <c r="C25" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="J24" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K24" s="2" t="s">
+      <c r="D25" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="F25" s="4" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="25" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="2" t="s">
+      <c r="G25" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="H25" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="I25" s="5"/>
+      <c r="J25" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K25" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="D25" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="F25" s="2" t="s">
+    </row>
+    <row r="26" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="G25" s="2" t="s">
+      <c r="B26" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="H25" s="2" t="s">
+      <c r="C26" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="J25" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K25" s="2" t="s">
+      <c r="D26" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E26" s="4" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="26" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="2" t="s">
+      <c r="F26" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="G26" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="H26" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="D26" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E26" s="2" t="s">
+      <c r="I26" s="5"/>
+      <c r="J26" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K26" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="F26" s="2" t="s">
+    </row>
+    <row r="27" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="G26" s="2" t="s">
+      <c r="B27" s="4" t="s">
         <v>204</v>
       </c>
-      <c r="H26" s="2" t="s">
+      <c r="C27" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="J26" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K26" s="2" t="s">
+      <c r="D27" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" s="4" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="27" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="2" t="s">
+      <c r="F27" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="G27" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="H27" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="D27" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E27" s="2" t="s">
+      <c r="I27" s="5"/>
+      <c r="J27" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K27" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="F27" s="2" t="s">
+    </row>
+    <row r="28" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="G27" s="2" t="s">
+      <c r="B28" s="4" t="s">
         <v>212</v>
       </c>
-      <c r="H27" s="2" t="s">
+      <c r="C28" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="J27" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K27" s="2" t="s">
+      <c r="D28" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" s="4" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="28" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="2" t="s">
+      <c r="F28" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="G28" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="H28" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="D28" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E28" s="2" t="s">
+      <c r="I28" s="5"/>
+      <c r="J28" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K28" s="6" t="s">
         <v>218</v>
       </c>
-      <c r="F28" s="2" t="s">
+    </row>
+    <row r="29" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="G28" s="2" t="s">
+      <c r="B29" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="H28" s="2" t="s">
+      <c r="C29" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="J28" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K28" s="2" t="s">
+      <c r="D29" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E29" s="4" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="29" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="2" t="s">
+      <c r="F29" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="G29" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="H29" s="4" t="s">
         <v>225</v>
       </c>
-      <c r="D29" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E29" s="2" t="s">
+      <c r="I29" s="5"/>
+      <c r="J29" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K29" s="6" t="s">
         <v>226</v>
       </c>
-      <c r="F29" s="2" t="s">
+    </row>
+    <row r="30" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="G29" s="2" t="s">
+      <c r="B30" s="4" t="s">
         <v>228</v>
       </c>
-      <c r="H29" s="2" t="s">
+      <c r="C30" s="4" t="s">
         <v>229</v>
       </c>
-      <c r="J29" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K29" s="2" t="s">
+      <c r="D30" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E30" s="4" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="30" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="2" t="s">
+      <c r="F30" s="4" t="s">
         <v>231</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="G30" s="4" t="s">
         <v>232</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="H30" s="4" t="s">
         <v>233</v>
       </c>
-      <c r="D30" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E30" s="2" t="s">
+      <c r="I30" s="5"/>
+      <c r="J30" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K30" s="6" t="s">
         <v>234</v>
       </c>
-      <c r="F30" s="2" t="s">
+    </row>
+    <row r="31" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="G30" s="2" t="s">
+      <c r="B31" s="8" t="s">
         <v>236</v>
       </c>
-      <c r="H30" s="2" t="s">
+      <c r="C31" s="8" t="s">
         <v>237</v>
       </c>
-      <c r="J30" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K30" s="2" t="s">
+      <c r="D31" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E31" s="8" t="s">
         <v>238</v>
       </c>
-    </row>
-    <row r="31" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="2" t="s">
+      <c r="F31" s="8" t="s">
         <v>239</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="G31" s="8" t="s">
         <v>240</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="H31" s="8" t="s">
         <v>241</v>
       </c>
-      <c r="D31" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E31" s="2" t="s">
+      <c r="I31" s="9"/>
+      <c r="J31" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="K31" s="10" t="s">
         <v>242</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="H31" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="J31" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K31" s="2" t="s">
-        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -2121,8 +2620,9 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>